<commit_message>
create csv files instead of xlsx files
</commit_message>
<xml_diff>
--- a/Outputs/Scenarios/PtX_demand_EU27_Ammonia.xlsx
+++ b/Outputs/Scenarios/PtX_demand_EU27_Ammonia.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,7 +498,7 @@
         <v>0.3423743809468868</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5628816558852643</v>
+        <v>0.5628816558852644</v>
       </c>
       <c r="E2" t="n">
         <v>0.04716776709385712</v>
@@ -572,7 +572,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06384674424382113</v>
+        <v>0.06384674424382114</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -967,157 +967,153 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Overall Demand</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
         <v>2030</v>
       </c>
       <c r="C15" t="n">
-        <v>0.8191346513205151</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8873450719697543</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0.80636152109936</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>5.837456875439707</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2540272909193773</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1.517999109009769</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>3.966611000776768</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1250793165508621</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>2.047540194129764</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Overall Demand</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2040</v>
+        <v>2030</v>
       </c>
       <c r="C16" t="n">
-        <v>0.3068326462227793</v>
+        <v>0.8191346513205151</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5204663086520501</v>
+        <v>0.8873450719697543</v>
       </c>
       <c r="E16" t="n">
-        <v>0.09434440816047998</v>
+        <v>0.80636152109936</v>
       </c>
       <c r="F16" t="n">
-        <v>0.8373860384421418</v>
+        <v>5.837456875439707</v>
       </c>
       <c r="G16" t="n">
-        <v>0.255577808831391</v>
+        <v>0.2540272909193773</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1.517999109009769</v>
       </c>
       <c r="I16" t="n">
-        <v>0.5220444296034016</v>
+        <v>3.966611000776768</v>
       </c>
       <c r="J16" t="n">
-        <v>0.07627629188289811</v>
+        <v>0.1250793165508621</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1281373516714958</v>
+        <v>2.047540194129764</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2040</v>
       </c>
       <c r="C17" t="n">
-        <v>0.08849981836020662</v>
+        <v>0.3068326462227793</v>
       </c>
       <c r="D17" t="n">
-        <v>0.04490295523796037</v>
+        <v>0.5204663086520501</v>
       </c>
       <c r="E17" t="n">
-        <v>0.03094661697621482</v>
+        <v>0.09434440816047998</v>
       </c>
       <c r="F17" t="n">
-        <v>0.02392608422744445</v>
+        <v>0.8373860384421418</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>0.255577808831391</v>
       </c>
       <c r="H17" t="n">
-        <v>9.424114493064826e-08</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.05492795755849274</v>
+        <v>0.5220444296034016</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>0.07627629188289811</v>
       </c>
       <c r="K17" t="n">
-        <v>0.02384419117424436</v>
+        <v>0.1281373516714958</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Methanol</t>
+          <t>Hydrogen</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2040</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.08849981836020662</v>
       </c>
       <c r="D18" t="n">
-        <v>0.05903564088222234</v>
+        <v>0.04490295523796037</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>0.03094661697621482</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>0.02392608422744445</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>9.424114493064826e-08</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>0.05492795755849274</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>0.02384419117424436</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Methanol</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1127,10 +1123,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.24097818031175</v>
+        <v>0.05903564088222234</v>
       </c>
       <c r="E19" t="n">
-        <v>0.006189323395242963</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -1148,13 +1144,13 @@
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1907535293939549</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Synthetic Gases</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1164,10 +1160,10 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>0.24097818031175</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>0.006189323395242963</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1185,13 +1181,13 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>0.1907535293939549</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Biogenic Gases</t>
+          <t>Synthetic Gases</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1204,10 +1200,10 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0.02162023123173737</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.003170713106672354</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1216,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.001484022904732818</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1228,7 +1224,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fossil Gases</t>
+          <t>Biogenic Gases</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1241,10 +1237,10 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>0.02162023123173737</v>
       </c>
       <c r="F22" t="n">
-        <v>0.04568464364411801</v>
+        <v>0.003170713106672354</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1253,7 +1249,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0.005770461290591195</v>
+        <v>0.001484022904732818</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -1265,7 +1261,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Synthetic Liquids</t>
+          <t>Fossil Gases</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1281,16 +1277,16 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>0.04568464364411801</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0.2433775467767053</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>0.005770461290591195</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -1302,7 +1298,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Biogenic Liquids</t>
+          <t>Synthetic Liquids</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1318,28 +1314,28 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2129621301111229</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0050009284501574</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1210971783029641</v>
+        <v>0.2433775467767053</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2710935229027119</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.00611279625632115</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.155829757115629</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Fossil Liquids</t>
+          <t>Biogenic Liquids</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1355,78 +1351,78 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>2.163554948828715</v>
+        <v>0.2129621301111229</v>
       </c>
       <c r="G25" t="n">
-        <v>0.03522007257660857</v>
+        <v>0.0050009284501574</v>
       </c>
       <c r="H25" t="n">
-        <v>1.090838846153271</v>
+        <v>0.1210971783029641</v>
       </c>
       <c r="I25" t="n">
-        <v>1.722317658292452</v>
+        <v>0.2710935229027119</v>
       </c>
       <c r="J25" t="n">
-        <v>0.03700076859972957</v>
+        <v>0.00611279625632115</v>
       </c>
       <c r="K25" t="n">
-        <v>1.487064521139202</v>
+        <v>0.155829757115629</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fossil Residuals</t>
+          <t>Fossil Liquids</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>2040</v>
       </c>
       <c r="C26" t="n">
-        <v>0.3143910666708016</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3514287196614972</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>2.163554948828715</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>0.03522007257660857</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1.090838846153271</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1.722317658292452</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>0.03700076859972957</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1.487064521139202</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Biomass [Solid]</t>
+          <t>Fossil Residuals</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2040</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>0.3143910666708016</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1318449308774697</v>
+        <v>0.3514287196614972</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1450,229 +1446,225 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Renewable Energy Carrier</t>
+          <t>Biomass [Solid]</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>2040</v>
       </c>
       <c r="C28" t="n">
-        <v>0.02678373880950322</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>0.02993530349197358</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>0.04218469786717863</v>
+        <v>0.1318449308774697</v>
       </c>
       <c r="F28" t="n">
-        <v>0.01808623629826565</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.00108317703936906</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>0.02704194964185614</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0.02372777619606962</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0.001099012251924778</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>0.02384419117424436</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Overall Demand</t>
+          <t>Renewable Energy Carrier</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2040</v>
       </c>
       <c r="C29" t="n">
-        <v>0.7365072700632906</v>
+        <v>0.02678373880950322</v>
       </c>
       <c r="D29" t="n">
-        <v>0.8953183885759565</v>
+        <v>0.02993530349197358</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6785589281698208</v>
+        <v>0.04218469786717863</v>
       </c>
       <c r="F29" t="n">
-        <v>3.30477079465848</v>
+        <v>0.01808623629826565</v>
       </c>
       <c r="G29" t="n">
-        <v>0.296881986897526</v>
+        <v>0.00108317703936906</v>
       </c>
       <c r="H29" t="n">
-        <v>1.482355615115942</v>
+        <v>0.02704194964185614</v>
       </c>
       <c r="I29" t="n">
-        <v>2.601365828748451</v>
+        <v>0.02372777619606962</v>
       </c>
       <c r="J29" t="n">
-        <v>0.1204888689908736</v>
+        <v>0.001099012251924778</v>
       </c>
       <c r="K29" t="n">
-        <v>2.009473541668771</v>
+        <v>0.02384419117424436</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>2050</v>
+        <v>2040</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2686123322676067</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>0.3819848435745393</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2759852536166209</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>2.107192483073658</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3236955155965828</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>1.319957314733273</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0.112917763768752</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>0.6881179361248416</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Hydrogen</t>
+          <t>Overall Demand</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2050</v>
+        <v>2040</v>
       </c>
       <c r="C31" t="n">
-        <v>0.2570632399817906</v>
+        <v>0.7365072700632906</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1806520242589478</v>
+        <v>0.8953183885759565</v>
       </c>
       <c r="E31" t="n">
-        <v>0.1379926268083105</v>
+        <v>0.6785589281698208</v>
       </c>
       <c r="F31" t="n">
-        <v>0.04436194701207702</v>
+        <v>3.30477079465848</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>0.296881986897526</v>
       </c>
       <c r="H31" t="n">
-        <v>8.9058142483003e-08</v>
+        <v>1.482355615115942</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1552890958509733</v>
+        <v>2.601365828748451</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>0.1204888689908736</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1280470948194029</v>
+        <v>2.009473541668771</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Methanol</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>2050</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>0.2686123322676067</v>
       </c>
       <c r="D32" t="n">
-        <v>0.04332791512696035</v>
+        <v>0.3819848435745392</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>0.2759852536166209</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>2.107192483073658</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>0.3236955155965828</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1.319957314733273</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>0.112917763768752</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>0.6881179361248416</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Hydrogen</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>2050</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>0.2570632399817906</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1768606554949931</v>
+        <v>0.1806520242589478</v>
       </c>
       <c r="E33" t="n">
-        <v>0.02759852536166209</v>
+        <v>0.1379926268083105</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>0.04436194701207702</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>8.9058142483003e-08</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>0.1552890958509733</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>1.024376758555223</v>
+        <v>0.1280470948194029</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Synthetic Gases</t>
+          <t>Methanol</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1682,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>0.04332791512696034</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -1709,7 +1701,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Biogenic Gases</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1719,10 +1711,10 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>0.176860655494993</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>0.02759852536166209</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -1740,13 +1732,13 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1.024376758555223</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Fossil Gases</t>
+          <t>Synthetic Gases</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1783,7 +1775,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Synthetic Liquids</t>
+          <t>Biogenic Gases</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1805,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1.260747124122744</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -1820,7 +1812,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Biogenic Liquids</t>
+          <t>Fossil Gases</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1857,7 +1849,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Fossil Liquids</t>
+          <t>Synthetic Liquids</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1879,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1.260747124122744</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -1894,7 +1886,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Fossil Residuals</t>
+          <t>Biogenic Liquids</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1931,7 +1923,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Biomass [Solid]</t>
+          <t>Fossil Liquids</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1968,74 +1960,181 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Renewable Energy Carrier</t>
+          <t>Fossil Residuals</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>2050</v>
       </c>
       <c r="C42" t="n">
-        <v>0.1285316199908953</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1204346828392985</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1103941014466484</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.06654292051811553</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0.006606030930542506</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.1400830137914161</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0.07764454792548665</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0.00594304019835537</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>0.1280470948194029</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Overall Demand</t>
+          <t>Biomass [Solid]</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>2050</v>
       </c>
       <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Renewable Energy Carrier</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2050</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.1285316199908953</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.1204346828392985</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.1103941014466484</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.06654292051811553</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.006606030930542506</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.1400830137914161</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.07764454792548665</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.00594304019835537</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.1280470948194029</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="n">
+        <v>2050</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Overall Demand</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2050</v>
+      </c>
+      <c r="C46" t="n">
         <v>0.6542071922402926</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D46" t="n">
         <v>0.903260121294739</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E46" t="n">
         <v>0.5519705072332418</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F46" t="n">
         <v>2.218097350603851</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G46" t="n">
         <v>0.3303015465271253</v>
       </c>
-      <c r="H43" t="n">
+      <c r="H46" t="n">
         <v>1.400830226972303</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I46" t="n">
         <v>1.552890958509733</v>
       </c>
-      <c r="J43" t="n">
+      <c r="J46" t="n">
         <v>0.1188608039671074</v>
       </c>
-      <c r="K43" t="n">
+      <c r="K46" t="n">
         <v>1.968588884318871</v>
       </c>
     </row>

</xml_diff>